<commit_message>
fix: keep R_ANALYSIS_FAILED visible on Vercel and lock the sample workbook
Live www treated worker 500 R_ANALYSIS_FAILED as a 502 unavailable copy, and the client had no mapping for that code. Forward a bounded detail excerpt, show analysis-failed in the browser, and generate the public Likert+Gender sample from the same helper analyze.R accepts.

Co-authored-by: Dr. Peter, Dongpin HU <HUDongpin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/open-sna/programming-resilience-sample.xlsx
+++ b/public/open-sna/programming-resilience-sample.xlsx
@@ -1,420 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:Q51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -505,52 +100,52 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
         <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N2" t="n">
         <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -560,52 +155,52 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
         <v>4</v>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -615,52 +210,52 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
         <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -670,34 +265,34 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
         <v>4</v>
@@ -706,13 +301,13 @@
         <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P5" t="n">
         <v>4</v>
@@ -725,52 +320,52 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -783,49 +378,49 @@
         <v>1</v>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O7" t="n">
         <v>5</v>
       </c>
       <c r="P7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -838,49 +433,49 @@
         <v>2</v>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
         <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -890,52 +485,52 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B9" t="n">
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -945,52 +540,52 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="n">
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
         <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M10" t="n">
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O10" t="n">
         <v>3</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1000,52 +595,52 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1055,52 +650,52 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
         <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1110,52 +705,52 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1165,34 +760,34 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
         <v>3</v>
@@ -1201,16 +796,16 @@
         <v>4</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
         <v>2</v>
       </c>
       <c r="P14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1220,52 +815,52 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J15" t="n">
         <v>3</v>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1278,22 +873,22 @@
         <v>5</v>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
@@ -1302,25 +897,25 @@
         <v>3</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1333,31 +928,31 @@
         <v>1</v>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
         <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
         <v>4</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K17" t="n">
         <v>1</v>
@@ -1366,16 +961,16 @@
         <v>2</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O17" t="n">
         <v>5</v>
       </c>
       <c r="P17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1385,46 +980,46 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I18" t="n">
         <v>5</v>
       </c>
       <c r="J18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N18" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O18" t="n">
         <v>1</v>
@@ -1440,52 +1035,52 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
         <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>3</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H19" t="n">
         <v>5</v>
       </c>
       <c r="I19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O19" t="n">
         <v>2</v>
       </c>
       <c r="P19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1498,49 +1093,49 @@
         <v>4</v>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -1550,19 +1145,19 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>5</v>
@@ -1571,31 +1166,31 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>3</v>
       </c>
       <c r="J21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
         <v>5</v>
       </c>
       <c r="L21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -1608,49 +1203,49 @@
         <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -1663,49 +1258,49 @@
         <v>2</v>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
         <v>5</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
         <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -1715,49 +1310,49 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
         <v>4</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M24" t="n">
         <v>5</v>
       </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P24" t="n">
         <v>3</v>
@@ -1770,28 +1365,28 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B25" t="n">
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
@@ -1800,22 +1395,22 @@
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O25" t="n">
         <v>3</v>
       </c>
       <c r="P25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -1825,52 +1420,52 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
         <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P26" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -1880,49 +1475,49 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P27" t="n">
         <v>1</v>
@@ -1935,52 +1530,52 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J28" t="n">
         <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -1993,43 +1588,43 @@
         <v>3</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
         <v>5</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K29" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
         <v>5</v>
       </c>
       <c r="N29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
         <v>2</v>
@@ -2051,46 +1646,46 @@
         <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
         <v>5</v>
       </c>
       <c r="M30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -2100,10 +1695,10 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
         <v>2</v>
@@ -2115,37 +1710,37 @@
         <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
         <v>2</v>
       </c>
       <c r="N31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -2155,34 +1750,34 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
@@ -2191,16 +1786,16 @@
         <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O32" t="n">
         <v>5</v>
       </c>
       <c r="P32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -2213,49 +1808,49 @@
         <v>2</v>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>2</v>
       </c>
       <c r="G33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I33" t="n">
         <v>5</v>
       </c>
       <c r="J33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -2265,52 +1860,52 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>3</v>
       </c>
       <c r="G34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -2323,19 +1918,19 @@
         <v>4</v>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G35" t="n">
         <v>5</v>
@@ -2344,28 +1939,28 @@
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>2</v>
       </c>
       <c r="O35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -2381,46 +1976,46 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
         <v>4</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -2430,52 +2025,52 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B37" t="n">
         <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
         <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K37" t="n">
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M37" t="n">
         <v>3</v>
       </c>
       <c r="N37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -2485,49 +2080,49 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
         <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P38" t="n">
         <v>2</v>
@@ -2543,43 +2138,43 @@
         <v>3</v>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" t="n">
         <v>5</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M39" t="n">
         <v>5</v>
       </c>
       <c r="N39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O39" t="n">
         <v>2</v>
@@ -2595,52 +2190,52 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
         <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L40" t="n">
         <v>5</v>
       </c>
       <c r="M40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -2653,49 +2248,49 @@
         <v>5</v>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E41" t="n">
         <v>4</v>
       </c>
       <c r="F41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J41" t="n">
         <v>4</v>
       </c>
       <c r="K41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O41" t="n">
         <v>4</v>
       </c>
       <c r="P41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -2705,43 +2300,43 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42" t="n">
         <v>5</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
         <v>5</v>
       </c>
       <c r="K42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
         <v>4</v>
@@ -2750,7 +2345,7 @@
         <v>5</v>
       </c>
       <c r="P42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -2766,46 +2361,46 @@
         <v>3</v>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H43" t="n">
         <v>4</v>
       </c>
       <c r="I43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -2815,49 +2410,49 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M44" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P44" t="n">
         <v>3</v>
@@ -2873,19 +2468,19 @@
         <v>4</v>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G45" t="n">
         <v>5</v>
@@ -2894,28 +2489,28 @@
         <v>1</v>
       </c>
       <c r="I45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L45" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M45" t="n">
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P45" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -2928,46 +2523,46 @@
         <v>5</v>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>5</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H46" t="n">
         <v>2</v>
       </c>
       <c r="I46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P46" t="n">
         <v>5</v>
@@ -2980,52 +2575,52 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K47" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>2</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -3035,37 +2630,37 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B48" t="n">
         <v>3</v>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G48" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
@@ -3074,10 +2669,10 @@
         <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P48" t="n">
         <v>2</v>
@@ -3090,49 +2685,49 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C49" t="n">
         <v>5</v>
       </c>
       <c r="D49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P49" t="n">
         <v>3</v>
@@ -3148,7 +2743,7 @@
         <v>4</v>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
@@ -3160,16 +2755,16 @@
         <v>3</v>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J50" t="n">
         <v>3</v>
@@ -3178,19 +2773,19 @@
         <v>4</v>
       </c>
       <c r="L50" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
@@ -3200,52 +2795,52 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>5</v>
       </c>
       <c r="G51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
         <v>3</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K51" t="n">
         <v>5</v>
       </c>
       <c r="L51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O51" t="n">
         <v>4</v>
       </c>
       <c r="P51" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
@@ -3254,6 +2849,5 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: condition Open SNA bootnet stability like the main NPN estimator
The published sample used cyclic Likert columns, so NPN correlations were
singular. Main/NCT already clipped eigenvalues, but bootnet's default npn
path stopped after NCT. Reuse the conditioned estimator for stability and
replace the sample with unique construct-factor Likert data.

Co-authored-by: Dr. Peter, Dongpin HU <HUDongpin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/open-sna/programming-resilience-sample.xlsx
+++ b/public/open-sna/programming-resilience-sample.xlsx
@@ -103,49 +103,49 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2" t="n">
         <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N2" t="n">
         <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -155,10 +155,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
         <v>4</v>
@@ -167,37 +167,37 @@
         <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K3" t="n">
         <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
@@ -210,52 +210,52 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -268,49 +268,49 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
         <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O5" t="n">
         <v>3</v>
       </c>
       <c r="P5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -320,10 +320,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
@@ -335,34 +335,34 @@
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P6" t="n">
         <v>5</v>
@@ -375,40 +375,40 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7" t="n">
         <v>3</v>
@@ -417,10 +417,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -436,46 +436,46 @@
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
         <v>3</v>
       </c>
       <c r="M8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -485,49 +485,49 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" t="n">
         <v>3</v>
@@ -540,13 +540,13 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10" t="n">
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -555,37 +555,37 @@
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M10" t="n">
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" t="n">
         <v>3</v>
       </c>
       <c r="P10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
@@ -604,43 +604,43 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
         <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O11" t="n">
         <v>4</v>
       </c>
       <c r="P11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -650,40 +650,40 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I12" t="n">
         <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
         <v>3</v>
@@ -692,10 +692,10 @@
         <v>4</v>
       </c>
       <c r="O12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -708,46 +708,46 @@
         <v>2</v>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13" t="n">
         <v>5</v>
       </c>
       <c r="O13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P13" t="n">
         <v>2</v>
@@ -766,46 +766,46 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K14" t="n">
         <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -815,13 +815,13 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
@@ -833,34 +833,34 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L15" t="n">
         <v>5</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -873,49 +873,49 @@
         <v>5</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
         <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -925,52 +925,52 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
         <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>2</v>
       </c>
       <c r="M17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -980,52 +980,52 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B18" t="n">
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
         <v>3</v>
       </c>
       <c r="M18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1035,43 +1035,43 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N19" t="n">
         <v>1</v>
@@ -1080,7 +1080,7 @@
         <v>2</v>
       </c>
       <c r="P19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1090,49 +1090,49 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K20" t="n">
         <v>4</v>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N20" t="n">
         <v>2</v>
       </c>
       <c r="O20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" t="n">
         <v>4</v>
@@ -1145,49 +1145,49 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P21" t="n">
         <v>5</v>
@@ -1200,19 +1200,19 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
@@ -1221,31 +1221,31 @@
         <v>2</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B23" t="n">
         <v>3</v>
@@ -1264,40 +1264,40 @@
         <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
         <v>3</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23" t="n">
         <v>5</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
@@ -1313,49 +1313,49 @@
         <v>3</v>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
         <v>4</v>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -1365,28 +1365,28 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
@@ -1395,22 +1395,22 @@
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O25" t="n">
         <v>3</v>
       </c>
       <c r="P25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -1420,52 +1420,52 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -1475,25 +1475,25 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B27" t="n">
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H27" t="n">
         <v>3</v>
@@ -1505,22 +1505,22 @@
         <v>5</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N27" t="n">
         <v>4</v>
       </c>
       <c r="O27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -1530,52 +1530,52 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -1585,49 +1585,49 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K29" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P29" t="n">
         <v>3</v>
@@ -1640,40 +1640,40 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>4</v>
       </c>
       <c r="G30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -1682,10 +1682,10 @@
         <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -1695,52 +1695,52 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
         <v>5</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M31" t="n">
         <v>2</v>
       </c>
       <c r="N31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -1750,52 +1750,52 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N32" t="n">
         <v>4</v>
       </c>
       <c r="O32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -1805,52 +1805,52 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H33" t="n">
         <v>4</v>
       </c>
       <c r="I33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -1860,52 +1860,52 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="n">
         <v>4</v>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H34" t="n">
         <v>5</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -1915,10 +1915,10 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
         <v>1</v>
@@ -1927,40 +1927,40 @@
         <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I35" t="n">
         <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -1970,52 +1970,52 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
         <v>4</v>
       </c>
       <c r="F36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M36" t="n">
         <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -2025,52 +2025,52 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C37" t="n">
         <v>3</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -2080,40 +2080,40 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
         <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M38" t="n">
         <v>4</v>
@@ -2122,10 +2122,10 @@
         <v>5</v>
       </c>
       <c r="O38" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -2135,49 +2135,49 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B39" t="n">
         <v>4</v>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J39" t="n">
         <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P39" t="n">
         <v>3</v>
@@ -2190,52 +2190,52 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>4</v>
       </c>
       <c r="G40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I40" t="n">
         <v>2</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L40" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N40" t="n">
         <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -2245,13 +2245,13 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
@@ -2266,22 +2266,22 @@
         <v>1</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K41" t="n">
         <v>5</v>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N41" t="n">
         <v>3</v>
@@ -2290,7 +2290,7 @@
         <v>4</v>
       </c>
       <c r="P41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -2306,46 +2306,46 @@
         <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
         <v>5</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
       </c>
       <c r="H42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M42" t="n">
         <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -2355,10 +2355,10 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43" t="n">
         <v>4</v>
@@ -2367,40 +2367,40 @@
         <v>5</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H43" t="n">
         <v>4</v>
       </c>
       <c r="I43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
         <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -2413,10 +2413,10 @@
         <v>3</v>
       </c>
       <c r="B44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
         <v>1</v>
@@ -2425,37 +2425,37 @@
         <v>2</v>
       </c>
       <c r="F44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J44" t="n">
         <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N44" t="n">
         <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
@@ -2465,28 +2465,28 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45" t="n">
         <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I45" t="n">
         <v>2</v>
@@ -2495,22 +2495,22 @@
         <v>3</v>
       </c>
       <c r="K45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M45" t="n">
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -2520,52 +2520,52 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D46" t="n">
         <v>3</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K46" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N46" t="n">
         <v>3</v>
       </c>
       <c r="O46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
@@ -2575,52 +2575,52 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N47" t="n">
         <v>4</v>
       </c>
       <c r="O47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -2633,34 +2633,34 @@
         <v>2</v>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
       </c>
       <c r="H48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I48" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
@@ -2669,13 +2669,13 @@
         <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -2685,13 +2685,13 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
         <v>1</v>
@@ -2700,37 +2700,37 @@
         <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
@@ -2740,10 +2740,10 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
@@ -2758,34 +2758,34 @@
         <v>4</v>
       </c>
       <c r="G50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I50" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O50" t="n">
         <v>3</v>
       </c>
       <c r="P50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
@@ -2795,52 +2795,52 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>5</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J51" t="n">
         <v>4</v>
       </c>
       <c r="K51" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P51" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(open-sna): raise public sample construct loadings
EBICglasso at gamma 0.5 still returned an empty graph on the first unique-column sample. Stronger construct loadings keep 16 distinct Likert series.

Co-authored-by: Dr. Peter, Dongpin HU <HUDongpin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/open-sna/programming-resilience-sample.xlsx
+++ b/public/open-sna/programming-resilience-sample.xlsx
@@ -103,13 +103,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
@@ -118,7 +118,7 @@
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
         <v>3</v>
@@ -130,7 +130,7 @@
         <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
         <v>4</v>
@@ -155,10 +155,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>4</v>
@@ -182,13 +182,13 @@
         <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
         <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
         <v>3</v>
@@ -219,19 +219,19 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
         <v>5</v>
@@ -249,13 +249,13 @@
         <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -265,13 +265,13 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="n">
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -283,7 +283,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
@@ -298,7 +298,7 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M5" t="n">
         <v>3</v>
@@ -326,7 +326,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
         <v>3</v>
@@ -347,7 +347,7 @@
         <v>4</v>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
@@ -390,7 +390,7 @@
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -399,7 +399,7 @@
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -408,13 +408,13 @@
         <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" t="n">
         <v>3</v>
       </c>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" t="n">
         <v>3</v>
@@ -436,16 +436,16 @@
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
         <v>3</v>
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="O8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>3</v>
@@ -494,13 +494,13 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
@@ -512,7 +512,7 @@
         <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -521,7 +521,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
         <v>2</v>
@@ -549,13 +549,13 @@
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="n">
         <v>4</v>
@@ -570,7 +570,7 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
         <v>2</v>
@@ -628,7 +628,7 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M11" t="n">
         <v>3</v>
@@ -637,7 +637,7 @@
         <v>4</v>
       </c>
       <c r="O11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
@@ -665,13 +665,13 @@
         <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
         <v>4</v>
@@ -695,7 +695,7 @@
         <v>3</v>
       </c>
       <c r="P12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -714,13 +714,13 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
         <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
         <v>4</v>
@@ -750,7 +750,7 @@
         <v>4</v>
       </c>
       <c r="P13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -760,13 +760,13 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B14" t="n">
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
         <v>3</v>
@@ -781,13 +781,13 @@
         <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
         <v>3</v>
@@ -815,19 +815,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B15" t="n">
         <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>4</v>
@@ -854,13 +854,13 @@
         <v>5</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O15" t="n">
         <v>5</v>
       </c>
       <c r="P15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -879,19 +879,19 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
         <v>5</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" t="n">
         <v>4</v>
@@ -915,7 +915,7 @@
         <v>3</v>
       </c>
       <c r="P16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -940,22 +940,22 @@
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L17" t="n">
         <v>2</v>
@@ -970,7 +970,7 @@
         <v>3</v>
       </c>
       <c r="P17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -980,10 +980,10 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -998,34 +998,34 @@
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K18" t="n">
         <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O18" t="n">
         <v>2</v>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1044,13 +1044,13 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
         <v>3</v>
@@ -1062,10 +1062,10 @@
         <v>2</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L19" t="n">
         <v>3</v>
@@ -1096,37 +1096,37 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I20" t="n">
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" t="n">
         <v>2</v>
@@ -1135,7 +1135,7 @@
         <v>2</v>
       </c>
       <c r="P20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -1157,31 +1157,31 @@
         <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21" t="n">
         <v>3</v>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21" t="n">
         <v>5</v>
@@ -1215,7 +1215,7 @@
         <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
@@ -1239,7 +1239,7 @@
         <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O22" t="n">
         <v>4</v>
@@ -1267,19 +1267,19 @@
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H23" t="n">
         <v>3</v>
       </c>
       <c r="I23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J23" t="n">
         <v>4</v>
@@ -1294,7 +1294,7 @@
         <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O23" t="n">
         <v>4</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B24" t="n">
         <v>1</v>
@@ -1325,7 +1325,7 @@
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" t="n">
         <v>4</v>
@@ -1349,13 +1349,13 @@
         <v>4</v>
       </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O24" t="n">
         <v>3</v>
       </c>
       <c r="P24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -1368,10 +1368,10 @@
         <v>1</v>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
         <v>4</v>
@@ -1392,19 +1392,19 @@
         <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
         <v>2</v>
       </c>
       <c r="L25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M25" t="n">
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25" t="n">
         <v>3</v>
@@ -1420,7 +1420,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B26" t="n">
         <v>3</v>
@@ -1429,7 +1429,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -1438,10 +1438,10 @@
         <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I26" t="n">
         <v>2</v>
@@ -1450,13 +1450,13 @@
         <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L26" t="n">
         <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
         <v>4</v>
@@ -1481,13 +1481,13 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>2</v>
@@ -1499,7 +1499,7 @@
         <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J27" t="n">
         <v>5</v>
@@ -1517,7 +1517,7 @@
         <v>4</v>
       </c>
       <c r="O27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P27" t="n">
         <v>4</v>
@@ -1572,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P28" t="n">
         <v>3</v>
@@ -1588,7 +1588,7 @@
         <v>4</v>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
         <v>2</v>
@@ -1606,7 +1606,7 @@
         <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I29" t="n">
         <v>3</v>
@@ -1649,31 +1649,31 @@
         <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
         <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K30" t="n">
         <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -1722,13 +1722,13 @@
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
         <v>4</v>
       </c>
       <c r="L31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M31" t="n">
         <v>2</v>
@@ -1737,7 +1737,7 @@
         <v>4</v>
       </c>
       <c r="O31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P31" t="n">
         <v>2</v>
@@ -1750,16 +1750,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B32" t="n">
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>4</v>
@@ -1774,16 +1774,16 @@
         <v>5</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J32" t="n">
         <v>3</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M32" t="n">
         <v>4</v>
@@ -1792,10 +1792,10 @@
         <v>4</v>
       </c>
       <c r="O32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G33" t="n">
         <v>2</v>
@@ -1835,13 +1835,13 @@
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
         <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N33" t="n">
         <v>3</v>
@@ -1850,7 +1850,7 @@
         <v>2</v>
       </c>
       <c r="P33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B34" t="n">
         <v>4</v>
@@ -1872,7 +1872,7 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>4</v>
@@ -1893,7 +1893,7 @@
         <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M34" t="n">
         <v>2</v>
@@ -1936,7 +1936,7 @@
         <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" t="n">
         <v>2</v>
@@ -1945,13 +1945,13 @@
         <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>1</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="P35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -1982,19 +1982,19 @@
         <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G36" t="n">
         <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
         <v>3</v>
@@ -2003,7 +2003,7 @@
         <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
         <v>2</v>
@@ -2049,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J37" t="n">
         <v>3</v>
@@ -2058,7 +2058,7 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37" t="n">
         <v>1</v>
@@ -2089,16 +2089,16 @@
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>4</v>
       </c>
       <c r="G38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H38" t="n">
         <v>5</v>
@@ -2107,10 +2107,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L38" t="n">
         <v>2</v>
@@ -2138,19 +2138,19 @@
         <v>2</v>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39" t="n">
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -2162,7 +2162,7 @@
         <v>2</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
         <v>2</v>
@@ -2190,28 +2190,28 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C40" t="n">
         <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
         <v>3</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
         <v>2</v>
@@ -2220,7 +2220,7 @@
         <v>2</v>
       </c>
       <c r="K40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
         <v>2</v>
@@ -2232,10 +2232,10 @@
         <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -2254,7 +2254,7 @@
         <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
         <v>4</v>
@@ -2263,7 +2263,7 @@
         <v>5</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" t="n">
         <v>4</v>
@@ -2272,13 +2272,13 @@
         <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" t="n">
         <v>5</v>
       </c>
       <c r="L41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M41" t="n">
         <v>4</v>
@@ -2300,31 +2300,31 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B42" t="n">
         <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
         <v>5</v>
       </c>
       <c r="F42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" t="n">
         <v>4</v>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
         <v>4</v>
@@ -2333,19 +2333,19 @@
         <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O42" t="n">
         <v>4</v>
       </c>
       <c r="P42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -2388,7 +2388,7 @@
         <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M43" t="n">
         <v>3</v>
@@ -2397,7 +2397,7 @@
         <v>3</v>
       </c>
       <c r="O43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P43" t="n">
         <v>3</v>
@@ -2416,7 +2416,7 @@
         <v>2</v>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>1</v>
@@ -2431,7 +2431,7 @@
         <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
         <v>2</v>
@@ -2446,13 +2446,13 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
         <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P44" t="n">
         <v>2</v>
@@ -2465,7 +2465,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B45" t="n">
         <v>3</v>
@@ -2480,19 +2480,19 @@
         <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I45" t="n">
         <v>2</v>
       </c>
       <c r="J45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K45" t="n">
         <v>2</v>
@@ -2541,7 +2541,7 @@
         <v>2</v>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I46" t="n">
         <v>2</v>
@@ -2590,16 +2590,16 @@
         <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G47" t="n">
         <v>4</v>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J47" t="n">
         <v>3</v>
@@ -2611,7 +2611,7 @@
         <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N47" t="n">
         <v>4</v>
@@ -2633,7 +2633,7 @@
         <v>2</v>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C48" t="n">
         <v>1</v>
@@ -2645,16 +2645,16 @@
         <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J48" t="n">
         <v>3</v>
@@ -2669,10 +2669,10 @@
         <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P48" t="n">
         <v>3</v>
@@ -2706,7 +2706,7 @@
         <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
@@ -2740,13 +2740,13 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
         <v>2</v>
@@ -2770,10 +2770,10 @@
         <v>5</v>
       </c>
       <c r="K50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M50" t="n">
         <v>4</v>
@@ -2804,7 +2804,7 @@
         <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E51" t="n">
         <v>3</v>
@@ -2813,7 +2813,7 @@
         <v>5</v>
       </c>
       <c r="G51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H51" t="n">
         <v>4</v>
@@ -2828,7 +2828,7 @@
         <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M51" t="n">
         <v>3</v>
@@ -2837,7 +2837,7 @@
         <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P51" t="n">
         <v>2</v>

</xml_diff>